<commit_message>
Re-run with updated FCVA logic threshold standardized to past FCVAs rubrics.
</commit_message>
<xml_diff>
--- a/outputs/Exposure-rank-vs-N-exp-factors.xlsx
+++ b/outputs/Exposure-rank-vs-N-exp-factors.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\Caribbean-CVA\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2C03C8F-2605-4654-9A00-6AD9BF2C4D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{36A9827F-3E88-448F-8568-C7C9FE5F8288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30915" yWindow="360" windowWidth="28740" windowHeight="15585" xr2:uid="{58C10DF4-8314-49A4-97A7-F953617E5974}"/>
+    <workbookView xWindow="30945" yWindow="1530" windowWidth="20130" windowHeight="11805" xr2:uid="{58C10DF4-8314-49A4-97A7-F953617E5974}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -325,7 +326,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -550,7 +551,7 @@
                   <c:v>3.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.0380000000000003</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>3</c:v>
@@ -565,7 +566,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>4.3</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>3.9</c:v>
@@ -574,7 +575,7 @@
                   <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.048</c:v>
+                  <c:v>4.0999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>3</c:v>
@@ -592,19 +593,19 @@
                   <c:v>4.2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2.8</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.806</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.86599999999999999</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.946</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.91800000000000004</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0.9</c:v>
@@ -613,7 +614,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.0760000000000001</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1458,16 +1459,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>600807</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>189399</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>21980</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>6226</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>307730</xdr:colOff>
+      <xdr:colOff>337038</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>36999</xdr:rowOff>
+      <xdr:rowOff>44326</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1900,8 +1901,7 @@
         <v>4</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E3:E26" ca="1" si="0">D5 + (RANDBETWEEN(-100,100) / 500)</f>
-        <v>4.0380000000000003</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1986,7 +1986,7 @@
         <v>4</v>
       </c>
       <c r="E10">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2037,8 +2037,7 @@
         <v>4</v>
       </c>
       <c r="E13">
-        <f t="shared" ca="1" si="0"/>
-        <v>4.048</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2140,8 +2139,7 @@
         <v>3</v>
       </c>
       <c r="E19">
-        <f t="shared" ca="1" si="0"/>
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -2158,8 +2156,7 @@
         <v>3</v>
       </c>
       <c r="E20">
-        <f t="shared" ca="1" si="0"/>
-        <v>2.806</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2176,8 +2173,7 @@
         <v>1</v>
       </c>
       <c r="E21">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.86599999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2194,8 +2190,7 @@
         <v>2</v>
       </c>
       <c r="E22">
-        <f t="shared" ca="1" si="0"/>
-        <v>1.946</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -2212,8 +2207,7 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.91800000000000004</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -2264,8 +2258,7 @@
         <v>1</v>
       </c>
       <c r="E26">
-        <f t="shared" ca="1" si="0"/>
-        <v>1.0760000000000001</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>